<commit_message>
Live Katalog-Korrektur via Streamlit Data Editor
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -545,12 +545,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>X</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>